<commit_message>
Switch email order import to Sage Intacct Order Entry
The Sage 300 layout is replaced by NPH's Intacct Order Entry import
template (Sage-OrderEntry_Import_headers.csv). The script now fills
whatever columns the template has, produces the CSV that Intacct's
import screen requires alongside the Excel copy, and looks up the
Intacct customer ID in Customer_Map.xlsx, which the flow reads each run.

- Customer lookup by ID/code in the email, sender address, addresses in
  forwarded mail, sender domain, then customer name; ambiguous or unknown
  matches mark the order REVIEW
- Template has no QUANTITY column, so lines for more than one unit are
  flagged for review until QUANTITY is added
- Dimension IDs, transaction type, state, due-date rule and column
  mapping are settings in getConfig()
- README rewritten for the Intacct flow, with decisions to confirm

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012yQXRcQWNgD85diFLU6vJo
</commit_message>
<xml_diff>
--- a/power-automate/sage-oe-email-import/samples/OE_Import_SAMPLE.xlsx
+++ b/power-automate/sage-oe-email-import/samples/OE_Import_SAMPLE.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order_Details" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OrderEntry_Import" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -58,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,218 +429,194 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
-    <col width="37" customWidth="1" min="9" max="9"/>
-    <col width="53" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ORDUNIQ</t>
+          <t>TRANSACTIONTYPE</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>ORDNUMBER</t>
+          <t>DATE</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>CUSTOMER</t>
+          <t>GLPOSTINGDATE</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>SHIPTO</t>
+          <t>CUSTOMER_ID</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>PONUMBER</t>
+          <t>DATEDUE</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>ORDDATE</t>
+          <t>DEPARTMENTID</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>EXPDATE</t>
+          <t>LOCATIONID</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>REFERENCE</t>
+          <t>LINE</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>DESC</t>
+          <t>ITEMID</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>COMMENT</t>
+          <t>PRICE</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>REFERENCENO</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>CLASSID</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>MEMO</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sales Order</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>46311</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>C-1001</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>*** NEW ***</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>1200</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>WHSE2</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>LMP-103-BLK</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>45-10872</t>
         </is>
       </c>
-      <c r="F2" s="3" t="n">
-        <v>46311</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <v>46325</v>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>PO 45-10872 - new order</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Email order from rblack@example.com</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Call receiving 30 min before delivery &amp; use dock 4.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ORDUNIQ</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>LINENUM</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>LINETYPE</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>ITEM</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>QTYORDERED</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>ORDUNIT</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>A1-103/0</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>EA</t>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Fluorescent Desk Lamp, Black</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>1</v>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Sales Order</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>46311</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>46311</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>A1-105/0</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>1200</v>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>EA</t>
+          <t>C-1001</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>LMP-105</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>45-10872</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Halogen Desk Lamp</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Import every invoice line as quantity 1
NPH's order emails are invoices that never show quantities, so the
parser no longer needs a Qty column to find the line table: an item
column next to a description or amount (or a description next to an
amount) is enough, and an Amount/Total column becomes PRICE when there
is no unit-price column.

- Lines default to quantity 1 (defaultQuantity); a quantity other than 1
  in an email is still flagged, since it would under-bill
- Accounting-style negatives like ($50.00) import as -50
- Lines without an item ID are kept and flagged instead of dropped
- Samples, tests and README updated to quantity-free invoices

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012yQXRcQWNgD85diFLU6vJo
</commit_message>
<xml_diff>
--- a/power-automate/sage-oe-email-import/samples/OE_Import_SAMPLE.xlsx
+++ b/power-automate/sage-oe-email-import/samples/OE_Import_SAMPLE.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -440,12 +440,12 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="27" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -547,11 +547,11 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>LMP-103-BLK</t>
+          <t>INST-100</t>
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>45</v>
+        <v>1250</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
@@ -566,7 +566,7 @@
       <c r="M2" s="2" t="n"/>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Fluorescent Desk Lamp, Black</t>
+          <t>Installation - Building A</t>
         </is>
       </c>
     </row>
@@ -597,11 +597,11 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>LMP-105</t>
+          <t>MAINT-200</t>
         </is>
       </c>
       <c r="J3" s="4" t="n">
-        <v>3.25</v>
+        <v>480</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
@@ -616,7 +616,57 @@
       <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Halogen Desk Lamp</t>
+          <t>Quarterly maintenance, Q4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Sales Order</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>46311</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>46311</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>C-1001</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>46325</v>
+      </c>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>DISC-10</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>-50</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>45-10872</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Loyalty discount</t>
         </is>
       </c>
     </row>

</xml_diff>